<commit_message>
Vlookpup, left, right, mid, pivot table, upper, sumif
</commit_message>
<xml_diff>
--- a/Excel/Career Decisions.xlsx
+++ b/Excel/Career Decisions.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c3f59aaaf5f4e1f8/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c3f59aaaf5f4e1f8/Desktop/Data-analysis/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{F79F7DDB-C8CF-4C38-9E86-65686155672D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06E6DE27-7137-4C66-8224-3C3E34A93789}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{F79F7DDB-C8CF-4C38-9E86-65686155672D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90C242F6-18F8-4AA3-82C0-296CD08C5206}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9880A8FC-3114-40D6-9A30-C32C787321EF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{9880A8FC-3114-40D6-9A30-C32C787321EF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Career Decision" sheetId="1" r:id="rId1"/>
+    <sheet name="Interesting Loan" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Career Decisions</t>
   </si>
@@ -73,16 +74,70 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Loan A</t>
+  </si>
+  <si>
+    <t>Loan B</t>
+  </si>
+  <si>
+    <t>Loan C</t>
+  </si>
+  <si>
+    <t>Loan D</t>
+  </si>
+  <si>
+    <t>Principle</t>
+  </si>
+  <si>
+    <t>Interest</t>
+  </si>
+  <si>
+    <t>Months</t>
+  </si>
+  <si>
+    <t>Interest P</t>
+  </si>
+  <si>
+    <t>Total Loan Paid</t>
+  </si>
+  <si>
+    <t>Monthly Payment</t>
+  </si>
+  <si>
+    <t>ctrl + D</t>
+  </si>
+  <si>
+    <t>Fill Down</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_ [$₹-44E]* #,##0.00_ ;_ [$₹-44E]* \-#,##0.00_ ;_ [$₹-44E]* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -135,25 +190,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -177,6 +235,899 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Monthly Payments for 20000 rs</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Interesting Loan'!$C$2:$C$5</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.09</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.0000000000000007E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.06</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Interesting Loan'!$G$2:$G$5</c:f>
+              <c:numCache>
+                <c:formatCode>_ [$₹-44E]* #,##0.00_ ;_ [$₹-44E]* \-#,##0.00_ ;_ [$₹-44E]* "-"??_ ;_ @_ </c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1816.6666666666667</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1800</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1783.3333333333333</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1766.6666666666667</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9647-4FF0-9BB0-8143ADFB82EA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="64436400"/>
+        <c:axId val="64430640"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="64436400"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="64430640"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="64430640"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="_ [$₹-44E]* #,##0.00_ ;_ [$₹-44E]* \-#,##0.00_ ;_ [$₹-44E]* &quot;-&quot;??_ ;_ @_ " sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="64436400"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>624840</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F63C2C36-2856-E3F0-F0B2-BF315B78507E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -493,45 +1444,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>3</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="2">
         <v>5</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="3">
         <v>4</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="4">
         <v>3</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="11">
+      <c r="K3" s="5">
         <v>1</v>
       </c>
       <c r="L3" t="s">
@@ -539,41 +1487,41 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="1">
         <v>1</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="1">
         <f>B4*C$3</f>
         <v>3</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="2">
         <v>5</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="2">
         <f>D4*E$3</f>
         <v>25</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="3">
         <v>1</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="3">
         <f>F4*G$3</f>
         <v>4</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="4">
         <v>4</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="4">
         <f>H4*I$3</f>
         <v>12</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="5">
         <v>5</v>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="5">
         <f>J4*K$3</f>
         <v>5</v>
       </c>
@@ -583,41 +1531,41 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="1">
         <v>4</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="1">
         <f t="shared" ref="C5:E8" si="0">B5*C$3</f>
         <v>12</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="2">
         <v>4</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="3">
         <v>3</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="3">
         <f t="shared" ref="G5" si="1">F5*G$3</f>
         <v>12</v>
       </c>
-      <c r="H5" s="9">
+      <c r="H5" s="4">
         <v>2</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="4">
         <f t="shared" ref="I5:K5" si="2">H5*I$3</f>
         <v>6</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="5">
         <v>1</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="5">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
@@ -627,41 +1575,41 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="1">
         <v>5</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="1">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="2">
         <v>1</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="3">
         <v>5</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="3">
         <f t="shared" ref="G6" si="4">F6*G$3</f>
         <v>20</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="4">
         <v>3</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="4">
         <f t="shared" ref="I6:K6" si="5">H6*I$3</f>
         <v>9</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="5">
         <v>3</v>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="5">
         <f t="shared" si="5"/>
         <v>3</v>
       </c>
@@ -671,41 +1619,41 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="2">
         <v>5</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="3">
         <v>4</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="3">
         <f t="shared" ref="G7" si="6">F7*G$3</f>
         <v>16</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="4">
         <v>4</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="4">
         <f t="shared" ref="I7:K7" si="7">H7*I$3</f>
         <v>12</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="5">
         <v>3</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="5">
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
@@ -715,41 +1663,41 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="1">
         <v>3</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="1">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="2">
         <v>5</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="3">
         <v>2</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="3">
         <f t="shared" ref="G8" si="8">F8*G$3</f>
         <v>8</v>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="4">
         <v>2</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="4">
         <f t="shared" ref="I8:K8" si="9">H8*I$3</f>
         <v>6</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="5">
         <v>5</v>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="5">
         <f t="shared" si="9"/>
         <v>5</v>
       </c>
@@ -764,4 +1712,154 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83C198ED-33AD-4D69-AAF0-F3692BBBD35E}">
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="7">
+        <v>20000</v>
+      </c>
+      <c r="C2" s="8">
+        <v>0.09</v>
+      </c>
+      <c r="D2">
+        <v>12</v>
+      </c>
+      <c r="E2" s="9">
+        <f>B2*C2</f>
+        <v>1800</v>
+      </c>
+      <c r="F2" s="9">
+        <f>B2+E2</f>
+        <v>21800</v>
+      </c>
+      <c r="G2" s="9">
+        <f>F2/D2</f>
+        <v>1816.6666666666667</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="7">
+        <v>20000</v>
+      </c>
+      <c r="C3" s="8">
+        <v>0.08</v>
+      </c>
+      <c r="D3">
+        <v>12</v>
+      </c>
+      <c r="E3" s="9">
+        <f t="shared" ref="E3:E5" si="0">B3*C3</f>
+        <v>1600</v>
+      </c>
+      <c r="F3" s="9">
+        <f t="shared" ref="F3:F5" si="1">B3+E3</f>
+        <v>21600</v>
+      </c>
+      <c r="G3" s="9">
+        <f t="shared" ref="G3:G5" si="2">F3/D3</f>
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="7">
+        <v>20000</v>
+      </c>
+      <c r="C4" s="8">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D4">
+        <v>12</v>
+      </c>
+      <c r="E4" s="9">
+        <f t="shared" si="0"/>
+        <v>1400.0000000000002</v>
+      </c>
+      <c r="F4" s="9">
+        <f t="shared" si="1"/>
+        <v>21400</v>
+      </c>
+      <c r="G4" s="9">
+        <f t="shared" si="2"/>
+        <v>1783.3333333333333</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="7">
+        <v>20000</v>
+      </c>
+      <c r="C5" s="8">
+        <v>0.06</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
+      </c>
+      <c r="E5" s="9">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
+      <c r="F5" s="9">
+        <f t="shared" si="1"/>
+        <v>21200</v>
+      </c>
+      <c r="G5" s="9">
+        <f t="shared" si="2"/>
+        <v>1766.6666666666667</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>